<commit_message>
refactor: Clean up scores package to 7 essential files and remove all duplicates
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/نمرات_نهایی_نواحی.xlsx
+++ b/نمرات_نهایی_نواحی.xlsx
@@ -71,7 +71,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -100,18 +100,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
         <bgColor rgb="00FEE2E2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-        <bgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
-        <bgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
     <fill>
@@ -147,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -179,13 +167,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -568,7 +550,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>نمره نسرا (۷۰-۱۰۰)</t>
+          <t>نمره واقعی (۰-۱۰۰)</t>
         </is>
       </c>
     </row>
@@ -579,7 +561,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -589,7 +571,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -599,7 +581,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -609,7 +591,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -619,7 +601,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -629,7 +611,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -639,7 +621,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>85.8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -649,7 +631,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -659,7 +641,7 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -669,7 +651,7 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -679,7 +661,7 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -689,7 +671,7 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -699,7 +681,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -709,7 +691,7 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -719,7 +701,7 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>97.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -729,7 +711,7 @@
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -739,7 +721,7 @@
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -749,7 +731,7 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20">
@@ -759,7 +741,7 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -769,7 +751,7 @@
         </is>
       </c>
       <c r="B21" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -779,7 +761,7 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -789,7 +771,7 @@
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
@@ -799,7 +781,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -809,7 +791,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -819,7 +801,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
@@ -829,7 +811,7 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
@@ -839,7 +821,7 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -849,7 +831,7 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -859,7 +841,7 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -869,7 +851,7 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -879,7 +861,7 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33">
@@ -889,7 +871,7 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -919,7 +901,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>جدول مقایسه نمرات دوره ۲ ماهه در دو مقیاس واقعی (۰ تا ۱۰۰) و استاندارد نسرا (۷۰ تا ۱۰۰)</t>
+          <t>جدول مقایسه نمرات دوره ۶ ماهه در دو مقیاس واقعی (۰ تا ۱۰۰) و استاندارد نسرا (۷۰ تا ۱۰۰)</t>
         </is>
       </c>
     </row>
@@ -997,7 +979,7 @@
       </c>
       <c r="H4" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1015,7 @@
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1051,7 @@
       </c>
       <c r="H6" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1087,7 @@
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1123,7 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1159,7 @@
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1191,27 +1173,29 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>52.8</v>
+        <v>0</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>85.8</v>
-      </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>2</v>
+        <v>70</v>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>52.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>کسری: 1 از 2 ماه (عدم فعالیت در: مرداد 1405)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1231,7 @@
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1267,7 @@
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1303,7 @@
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1339,7 @@
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1375,7 @@
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1411,7 @@
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1463,7 +1447,7 @@
       </c>
       <c r="H17" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1477,27 +1461,29 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>90.8</v>
+        <v>0</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>97.2</v>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
-        <is>
-          <t>عالی</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>1</v>
+        <v>70</v>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>90.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="H18" s="10" t="inlineStr">
         <is>
-          <t>کامل (2 از 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1519,7 @@
       </c>
       <c r="H19" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1569,7 +1555,7 @@
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1591,7 @@
       </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1641,7 +1627,7 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1677,7 +1663,7 @@
       </c>
       <c r="H23" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1699,7 @@
       </c>
       <c r="H24" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1749,7 +1735,7 @@
       </c>
       <c r="H25" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1771,7 @@
       </c>
       <c r="H26" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1807,7 @@
       </c>
       <c r="H27" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1857,7 +1843,7 @@
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1893,7 +1879,7 @@
       </c>
       <c r="H29" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1915,7 @@
       </c>
       <c r="H30" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -1965,7 +1951,7 @@
       </c>
       <c r="H31" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2001,7 +1987,7 @@
       </c>
       <c r="H32" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2037,7 +2023,7 @@
       </c>
       <c r="H33" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2059,7 @@
       </c>
       <c r="H34" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2095,7 @@
       </c>
       <c r="H35" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2142,7 +2128,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>جدول ارزیابی عملکرد ۲ ماهه نواحی نسرا (مقیاس استاندارد نسرا (۷۰ تا ۱۰۰))</t>
+          <t>جدول ارزیابی عملکرد ۶ ماهه نواحی نسرا (مقیاس واقعی (۰ تا ۱۰۰))</t>
         </is>
       </c>
     </row>
@@ -2159,7 +2145,7 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>نمره نسرا (۷۰-۱۰۰)</t>
+          <t>نمره واقعی (۰-۱۰۰)</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -2193,7 +2179,7 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
@@ -2207,12 +2193,12 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G4" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2212,7 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
@@ -2240,12 +2226,12 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2245,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -2273,12 +2259,12 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2278,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
@@ -2306,12 +2292,12 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2311,7 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
@@ -2339,12 +2325,12 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2358,7 +2344,7 @@
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
@@ -2372,12 +2358,12 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2391,24 +2377,26 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>85.8</v>
-      </c>
-      <c r="D10" s="11" t="inlineStr">
-        <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>1 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>کسری: 1 از 2 ماه (عدم فعالیت در: مرداد 1405)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2410,7 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
@@ -2436,12 +2424,12 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2455,7 +2443,7 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
@@ -2469,12 +2457,12 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2476,7 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
@@ -2502,12 +2490,12 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2509,7 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
@@ -2535,12 +2523,12 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2542,7 @@
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -2568,12 +2556,12 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2587,7 +2575,7 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -2601,12 +2589,12 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2608,7 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -2634,12 +2622,12 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2653,24 +2641,26 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>97.2</v>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>عالی</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>2 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>کامل (2 از 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2684,7 +2674,7 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
@@ -2698,12 +2688,12 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2717,7 +2707,7 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
@@ -2731,12 +2721,12 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2750,7 +2740,7 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
@@ -2764,12 +2754,12 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2783,7 +2773,7 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
@@ -2797,12 +2787,12 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2816,7 +2806,7 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
@@ -2830,12 +2820,12 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2839,7 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
@@ -2863,12 +2853,12 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2872,7 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
@@ -2896,12 +2886,12 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2915,7 +2905,7 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D26" s="9" t="inlineStr">
         <is>
@@ -2929,12 +2919,12 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2948,7 +2938,7 @@
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
@@ -2962,12 +2952,12 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -2981,7 +2971,7 @@
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
@@ -2995,12 +2985,12 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -3014,7 +3004,7 @@
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
@@ -3028,12 +3018,12 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -3047,7 +3037,7 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
@@ -3061,12 +3051,12 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3070,7 @@
         </is>
       </c>
       <c r="C31" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
@@ -3094,12 +3084,12 @@
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -3113,7 +3103,7 @@
         </is>
       </c>
       <c r="C32" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D32" s="9" t="inlineStr">
         <is>
@@ -3127,12 +3117,12 @@
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -3146,7 +3136,7 @@
         </is>
       </c>
       <c r="C33" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -3160,12 +3150,12 @@
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G33" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -3179,7 +3169,7 @@
         </is>
       </c>
       <c r="C34" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -3193,12 +3183,12 @@
       </c>
       <c r="F34" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -3212,7 +3202,7 @@
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -3226,12 +3216,12 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
       <c r="G35" s="10" t="inlineStr">
         <is>
-          <t>فاقد گزارش (عملکرد ۰ در کل 2 ماه)</t>
+          <t>فاقد گزارش (عملکرد ۰ در کل 6 ماه)</t>
         </is>
       </c>
     </row>
@@ -3264,106 +3254,110 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>رتبه‌بندی استانی عملکرد ۲ ماهه ۳۲ شهرستان (مقیاس استاندارد نسرا (۷۰ تا ۱۰۰))</t>
+          <t>رتبه‌بندی استانی عملکرد ۶ ماهه ۳۲ شهرستان (مقیاس واقعی (۰ تا ۱۰۰))</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>رتبه</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>نام ناحیه (شهرستان)</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
-        <is>
-          <t>نمره نسرا (۷۰-۱۰۰)</t>
-        </is>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>نمره واقعی (۰-۱۰۰)</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>نمره مقیاس دیگر</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>سطح کیفی</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>درصد تحقق وزنی</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>تعداد ماه‌های ارسالی</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
-        <v>1</v>
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>درچه</t>
+          <t>آران و بیدگل</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>97.2</v>
+        <v>0</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>90.8</v>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>عالی</t>
+        <v>70</v>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>90.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>2 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
-        <v>2</v>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>برخوار</t>
+          <t>امام حسین(ع)</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>85.8</v>
+        <v>0</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>52.8</v>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>متوسط</t>
+        <v>70</v>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>ضعیف</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>52.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>1 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3375,14 +3369,14 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>آران و بیدگل</t>
+          <t>امام رضا(ع)</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
@@ -3396,7 +3390,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3408,14 +3402,14 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>امام حسین(ع)</t>
+          <t>امام صادق(ع)</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
@@ -3429,7 +3423,7 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3441,14 +3435,14 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>امام رضا(ع)</t>
+          <t>امام علی(ع)</t>
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
@@ -3462,7 +3456,7 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3474,14 +3468,14 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>امام صادق(ع)</t>
+          <t>اردستان</t>
         </is>
       </c>
       <c r="C9" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
@@ -3495,7 +3489,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3507,14 +3501,14 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>امام علی(ع)</t>
+          <t>برخوار</t>
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
@@ -3528,7 +3522,7 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3540,14 +3534,14 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>اردستان</t>
+          <t>بویین و میاندشت</t>
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
@@ -3561,7 +3555,7 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3573,14 +3567,14 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>بویین و میاندشت</t>
+          <t>تیران و کرون</t>
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
@@ -3594,7 +3588,7 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3606,14 +3600,14 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>تیران و کرون</t>
+          <t>جرقویه</t>
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
@@ -3627,7 +3621,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3639,14 +3633,14 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>جرقویه</t>
+          <t>چادگان</t>
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
@@ -3660,7 +3654,7 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3672,14 +3666,14 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>چادگان</t>
+          <t>خمینی شهر</t>
         </is>
       </c>
       <c r="C15" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
@@ -3693,7 +3687,7 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3705,14 +3699,14 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>خمینی شهر</t>
+          <t>خوانسار</t>
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
@@ -3726,7 +3720,7 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3738,14 +3732,14 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>خوانسار</t>
+          <t>خور و بیابانک</t>
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
@@ -3759,7 +3753,7 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3771,14 +3765,14 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>خور و بیابانک</t>
+          <t>درچه</t>
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
@@ -3792,7 +3786,7 @@
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3808,10 +3802,10 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
@@ -3825,7 +3819,7 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3841,10 +3835,10 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
@@ -3858,7 +3852,7 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3874,10 +3868,10 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
@@ -3891,7 +3885,7 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3907,10 +3901,10 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
@@ -3924,7 +3918,7 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3940,10 +3934,10 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
@@ -3957,7 +3951,7 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -3973,10 +3967,10 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
@@ -3990,7 +3984,7 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -4006,10 +4000,10 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
@@ -4023,7 +4017,7 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -4039,10 +4033,10 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
@@ -4056,7 +4050,7 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -4072,10 +4066,10 @@
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
@@ -4089,7 +4083,7 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -4105,10 +4099,10 @@
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
@@ -4122,7 +4116,7 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -4138,10 +4132,10 @@
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D29" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
@@ -4155,7 +4149,7 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -4171,10 +4165,10 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D30" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E30" s="9" t="inlineStr">
         <is>
@@ -4188,7 +4182,7 @@
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -4204,10 +4198,10 @@
         </is>
       </c>
       <c r="C31" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D31" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E31" s="9" t="inlineStr">
         <is>
@@ -4221,7 +4215,7 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -4237,10 +4231,10 @@
         </is>
       </c>
       <c r="C32" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
@@ -4254,7 +4248,7 @@
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -4270,10 +4264,10 @@
         </is>
       </c>
       <c r="C33" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E33" s="9" t="inlineStr">
         <is>
@@ -4287,7 +4281,7 @@
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -4303,10 +4297,10 @@
         </is>
       </c>
       <c r="C34" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E34" s="9" t="inlineStr">
         <is>
@@ -4320,7 +4314,7 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -4336,10 +4330,10 @@
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="E35" s="9" t="inlineStr">
         <is>
@@ -4353,7 +4347,7 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>0 از 2 ماه</t>
+          <t>0 از 6 ماه</t>
         </is>
       </c>
     </row>
@@ -4400,112 +4394,112 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>ریز مستندات و اوزان شاخص‌های دوره ۲ ماهه به تفکیک شهرستان‌ها</t>
+          <t>ریز مستندات و اوزان شاخص‌های دوره ۶ ماهه به تفکیک شهرستان‌ها</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>ردیف</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>نام ناحیه</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>نمره واقعی (۰-۱۰۰)</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>نمره نسرا (۷۰-۱۰۰)</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>سطح</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="F3" s="11" t="inlineStr">
         <is>
           <t>رتبه</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>ماه‌ها</t>
         </is>
       </c>
-      <c r="H3" s="13" t="inlineStr">
+      <c r="H3" s="11" t="inlineStr">
         <is>
           <t>حوزه</t>
         </is>
       </c>
-      <c r="I3" s="13" t="inlineStr">
+      <c r="I3" s="11" t="inlineStr">
         <is>
           <t>انتظار حضوری</t>
         </is>
       </c>
-      <c r="J3" s="13" t="inlineStr">
+      <c r="J3" s="11" t="inlineStr">
         <is>
           <t>عملکرد حضوری</t>
         </is>
       </c>
-      <c r="K3" s="13" t="inlineStr">
+      <c r="K3" s="11" t="inlineStr">
         <is>
           <t>تحقق حضوری</t>
         </is>
       </c>
-      <c r="L3" s="13" t="inlineStr">
+      <c r="L3" s="11" t="inlineStr">
         <is>
           <t>انتظار مجازی</t>
         </is>
       </c>
-      <c r="M3" s="13" t="inlineStr">
+      <c r="M3" s="11" t="inlineStr">
         <is>
           <t>عملکرد مجازی</t>
         </is>
       </c>
-      <c r="N3" s="13" t="inlineStr">
+      <c r="N3" s="11" t="inlineStr">
         <is>
           <t>تحقق مجازی</t>
         </is>
       </c>
-      <c r="O3" s="13" t="inlineStr">
+      <c r="O3" s="11" t="inlineStr">
         <is>
           <t>سهم آموزش (۴۰٪)</t>
         </is>
       </c>
-      <c r="P3" s="13" t="inlineStr">
+      <c r="P3" s="11" t="inlineStr">
         <is>
           <t>انتظار خلاقانه</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
+      <c r="Q3" s="11" t="inlineStr">
         <is>
           <t>عملکرد خلاقانه</t>
         </is>
       </c>
-      <c r="R3" s="13" t="inlineStr">
+      <c r="R3" s="11" t="inlineStr">
         <is>
           <t>سهم خلاقانه (۵۰٪)</t>
         </is>
       </c>
-      <c r="S3" s="13" t="inlineStr">
+      <c r="S3" s="11" t="inlineStr">
         <is>
           <t>انتظار تولید</t>
         </is>
       </c>
-      <c r="T3" s="13" t="inlineStr">
+      <c r="T3" s="11" t="inlineStr">
         <is>
           <t>عملکرد تولید</t>
         </is>
       </c>
-      <c r="U3" s="13" t="inlineStr">
+      <c r="U3" s="11" t="inlineStr">
         <is>
           <t>سهم تولید (۱۰٪)</t>
         </is>
@@ -4538,14 +4532,14 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H4" s="6" t="n">
         <v>10</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>620</v>
+        <v>1860</v>
       </c>
       <c r="J4" s="6" t="n">
         <v>0</v>
@@ -4556,7 +4550,7 @@
         </is>
       </c>
       <c r="L4" s="6" t="n">
-        <v>4340</v>
+        <v>13020</v>
       </c>
       <c r="M4" s="6" t="n">
         <v>0</v>
@@ -4572,7 +4566,7 @@
         </is>
       </c>
       <c r="P4" s="6" t="n">
-        <v>1240</v>
+        <v>3720</v>
       </c>
       <c r="Q4" s="6" t="n">
         <v>0</v>
@@ -4583,7 +4577,7 @@
         </is>
       </c>
       <c r="S4" s="6" t="n">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="T4" s="6" t="n">
         <v>0</v>
@@ -4621,14 +4615,14 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H5" s="6" t="n">
         <v>5</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>310</v>
+        <v>930</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>0</v>
@@ -4639,7 +4633,7 @@
         </is>
       </c>
       <c r="L5" s="6" t="n">
-        <v>2170</v>
+        <v>6510</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>0</v>
@@ -4655,7 +4649,7 @@
         </is>
       </c>
       <c r="P5" s="6" t="n">
-        <v>620</v>
+        <v>1860</v>
       </c>
       <c r="Q5" s="6" t="n">
         <v>0</v>
@@ -4666,7 +4660,7 @@
         </is>
       </c>
       <c r="S5" s="6" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="T5" s="6" t="n">
         <v>0</v>
@@ -4704,14 +4698,14 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H6" s="6" t="n">
         <v>22</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>1364</v>
+        <v>4092</v>
       </c>
       <c r="J6" s="6" t="n">
         <v>0</v>
@@ -4722,7 +4716,7 @@
         </is>
       </c>
       <c r="L6" s="6" t="n">
-        <v>9548</v>
+        <v>28644</v>
       </c>
       <c r="M6" s="6" t="n">
         <v>0</v>
@@ -4738,7 +4732,7 @@
         </is>
       </c>
       <c r="P6" s="6" t="n">
-        <v>2728</v>
+        <v>8184</v>
       </c>
       <c r="Q6" s="6" t="n">
         <v>0</v>
@@ -4749,7 +4743,7 @@
         </is>
       </c>
       <c r="S6" s="6" t="n">
-        <v>132</v>
+        <v>396</v>
       </c>
       <c r="T6" s="6" t="n">
         <v>0</v>
@@ -4787,14 +4781,14 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H7" s="6" t="n">
         <v>22</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>1364</v>
+        <v>4092</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>0</v>
@@ -4805,7 +4799,7 @@
         </is>
       </c>
       <c r="L7" s="6" t="n">
-        <v>9548</v>
+        <v>28644</v>
       </c>
       <c r="M7" s="6" t="n">
         <v>0</v>
@@ -4821,7 +4815,7 @@
         </is>
       </c>
       <c r="P7" s="6" t="n">
-        <v>2728</v>
+        <v>8184</v>
       </c>
       <c r="Q7" s="6" t="n">
         <v>0</v>
@@ -4832,7 +4826,7 @@
         </is>
       </c>
       <c r="S7" s="6" t="n">
-        <v>132</v>
+        <v>396</v>
       </c>
       <c r="T7" s="6" t="n">
         <v>0</v>
@@ -4870,14 +4864,14 @@
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H8" s="6" t="n">
         <v>6</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>372</v>
+        <v>1116</v>
       </c>
       <c r="J8" s="6" t="n">
         <v>0</v>
@@ -4888,7 +4882,7 @@
         </is>
       </c>
       <c r="L8" s="6" t="n">
-        <v>2604</v>
+        <v>7812</v>
       </c>
       <c r="M8" s="6" t="n">
         <v>0</v>
@@ -4904,7 +4898,7 @@
         </is>
       </c>
       <c r="P8" s="6" t="n">
-        <v>744</v>
+        <v>2232</v>
       </c>
       <c r="Q8" s="6" t="n">
         <v>0</v>
@@ -4915,7 +4909,7 @@
         </is>
       </c>
       <c r="S8" s="6" t="n">
-        <v>36</v>
+        <v>108</v>
       </c>
       <c r="T8" s="6" t="n">
         <v>0</v>
@@ -4953,14 +4947,14 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H9" s="6" t="n">
         <v>6</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>372</v>
+        <v>1116</v>
       </c>
       <c r="J9" s="6" t="n">
         <v>0</v>
@@ -4971,7 +4965,7 @@
         </is>
       </c>
       <c r="L9" s="6" t="n">
-        <v>2604</v>
+        <v>7812</v>
       </c>
       <c r="M9" s="6" t="n">
         <v>0</v>
@@ -4987,7 +4981,7 @@
         </is>
       </c>
       <c r="P9" s="6" t="n">
-        <v>744</v>
+        <v>2232</v>
       </c>
       <c r="Q9" s="6" t="n">
         <v>0</v>
@@ -4998,7 +4992,7 @@
         </is>
       </c>
       <c r="S9" s="6" t="n">
-        <v>36</v>
+        <v>108</v>
       </c>
       <c r="T9" s="6" t="n">
         <v>0</v>
@@ -5019,43 +5013,45 @@
         </is>
       </c>
       <c r="C10" s="7" t="n">
-        <v>52.8</v>
+        <v>0</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>85.8</v>
+        <v>70</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>متوسط</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>2</v>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>1 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H10" s="6" t="n">
         <v>5</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>310</v>
+        <v>930</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>14.8%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="L10" s="6" t="n">
-        <v>2170</v>
+        <v>6510</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N10" s="6" t="inlineStr">
         <is>
@@ -5064,29 +5060,29 @@
       </c>
       <c r="O10" s="6" t="inlineStr">
         <is>
-          <t>1.50%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P10" s="6" t="n">
-        <v>620</v>
+        <v>1860</v>
       </c>
       <c r="Q10" s="6" t="n">
-        <v>4396</v>
+        <v>0</v>
       </c>
       <c r="R10" s="6" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="S10" s="6" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="T10" s="6" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="U10" s="6" t="inlineStr">
         <is>
-          <t>1.33%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -5117,14 +5113,14 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H11" s="6" t="n">
         <v>3</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>186</v>
+        <v>558</v>
       </c>
       <c r="J11" s="6" t="n">
         <v>0</v>
@@ -5135,7 +5131,7 @@
         </is>
       </c>
       <c r="L11" s="6" t="n">
-        <v>1302</v>
+        <v>3906</v>
       </c>
       <c r="M11" s="6" t="n">
         <v>0</v>
@@ -5151,7 +5147,7 @@
         </is>
       </c>
       <c r="P11" s="6" t="n">
-        <v>372</v>
+        <v>1116</v>
       </c>
       <c r="Q11" s="6" t="n">
         <v>0</v>
@@ -5162,7 +5158,7 @@
         </is>
       </c>
       <c r="S11" s="6" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="T11" s="6" t="n">
         <v>0</v>
@@ -5200,14 +5196,14 @@
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H12" s="6" t="n">
         <v>6</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>372</v>
+        <v>1116</v>
       </c>
       <c r="J12" s="6" t="n">
         <v>0</v>
@@ -5218,7 +5214,7 @@
         </is>
       </c>
       <c r="L12" s="6" t="n">
-        <v>2604</v>
+        <v>7812</v>
       </c>
       <c r="M12" s="6" t="n">
         <v>0</v>
@@ -5234,7 +5230,7 @@
         </is>
       </c>
       <c r="P12" s="6" t="n">
-        <v>744</v>
+        <v>2232</v>
       </c>
       <c r="Q12" s="6" t="n">
         <v>0</v>
@@ -5245,7 +5241,7 @@
         </is>
       </c>
       <c r="S12" s="6" t="n">
-        <v>36</v>
+        <v>108</v>
       </c>
       <c r="T12" s="6" t="n">
         <v>0</v>
@@ -5283,14 +5279,14 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H13" s="6" t="n">
         <v>4</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>248</v>
+        <v>744</v>
       </c>
       <c r="J13" s="6" t="n">
         <v>0</v>
@@ -5301,7 +5297,7 @@
         </is>
       </c>
       <c r="L13" s="6" t="n">
-        <v>1736</v>
+        <v>5208</v>
       </c>
       <c r="M13" s="6" t="n">
         <v>0</v>
@@ -5317,7 +5313,7 @@
         </is>
       </c>
       <c r="P13" s="6" t="n">
-        <v>496</v>
+        <v>1488</v>
       </c>
       <c r="Q13" s="6" t="n">
         <v>0</v>
@@ -5328,7 +5324,7 @@
         </is>
       </c>
       <c r="S13" s="6" t="n">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="T13" s="6" t="n">
         <v>0</v>
@@ -5366,14 +5362,14 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H14" s="6" t="n">
         <v>5</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>310</v>
+        <v>930</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>0</v>
@@ -5384,7 +5380,7 @@
         </is>
       </c>
       <c r="L14" s="6" t="n">
-        <v>2170</v>
+        <v>6510</v>
       </c>
       <c r="M14" s="6" t="n">
         <v>0</v>
@@ -5400,7 +5396,7 @@
         </is>
       </c>
       <c r="P14" s="6" t="n">
-        <v>620</v>
+        <v>1860</v>
       </c>
       <c r="Q14" s="6" t="n">
         <v>0</v>
@@ -5411,7 +5407,7 @@
         </is>
       </c>
       <c r="S14" s="6" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="T14" s="6" t="n">
         <v>0</v>
@@ -5449,14 +5445,14 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H15" s="6" t="n">
         <v>9</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>558</v>
+        <v>1674</v>
       </c>
       <c r="J15" s="6" t="n">
         <v>0</v>
@@ -5467,7 +5463,7 @@
         </is>
       </c>
       <c r="L15" s="6" t="n">
-        <v>3906</v>
+        <v>11718</v>
       </c>
       <c r="M15" s="6" t="n">
         <v>0</v>
@@ -5483,7 +5479,7 @@
         </is>
       </c>
       <c r="P15" s="6" t="n">
-        <v>1116</v>
+        <v>3348</v>
       </c>
       <c r="Q15" s="6" t="n">
         <v>0</v>
@@ -5494,7 +5490,7 @@
         </is>
       </c>
       <c r="S15" s="6" t="n">
-        <v>54</v>
+        <v>162</v>
       </c>
       <c r="T15" s="6" t="n">
         <v>0</v>
@@ -5532,14 +5528,14 @@
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H16" s="6" t="n">
         <v>3</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>186</v>
+        <v>558</v>
       </c>
       <c r="J16" s="6" t="n">
         <v>0</v>
@@ -5550,7 +5546,7 @@
         </is>
       </c>
       <c r="L16" s="6" t="n">
-        <v>1302</v>
+        <v>3906</v>
       </c>
       <c r="M16" s="6" t="n">
         <v>0</v>
@@ -5566,7 +5562,7 @@
         </is>
       </c>
       <c r="P16" s="6" t="n">
-        <v>372</v>
+        <v>1116</v>
       </c>
       <c r="Q16" s="6" t="n">
         <v>0</v>
@@ -5577,7 +5573,7 @@
         </is>
       </c>
       <c r="S16" s="6" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="T16" s="6" t="n">
         <v>0</v>
@@ -5615,14 +5611,14 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H17" s="6" t="n">
         <v>2</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>124</v>
+        <v>372</v>
       </c>
       <c r="J17" s="6" t="n">
         <v>0</v>
@@ -5633,7 +5629,7 @@
         </is>
       </c>
       <c r="L17" s="6" t="n">
-        <v>868</v>
+        <v>2604</v>
       </c>
       <c r="M17" s="6" t="n">
         <v>0</v>
@@ -5649,7 +5645,7 @@
         </is>
       </c>
       <c r="P17" s="6" t="n">
-        <v>248</v>
+        <v>744</v>
       </c>
       <c r="Q17" s="6" t="n">
         <v>0</v>
@@ -5660,7 +5656,7 @@
         </is>
       </c>
       <c r="S17" s="6" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="T17" s="6" t="n">
         <v>0</v>
@@ -5681,74 +5677,76 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>90.8</v>
+        <v>0</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>97.2</v>
+        <v>70</v>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>عالی</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="n">
-        <v>1</v>
+          <t>ضعیف</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>2 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H18" s="6" t="n">
         <v>4</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>248</v>
+        <v>744</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>4552</v>
+        <v>0</v>
       </c>
       <c r="K18" s="6" t="inlineStr">
         <is>
-          <t>1835.5%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="L18" s="6" t="n">
-        <v>1736</v>
+        <v>5208</v>
       </c>
       <c r="M18" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N18" s="6" t="inlineStr">
         <is>
-          <t>0.1%</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="O18" s="6" t="inlineStr">
         <is>
-          <t>40.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="P18" s="6" t="n">
-        <v>496</v>
+        <v>1488</v>
       </c>
       <c r="Q18" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R18" s="6" t="inlineStr">
         <is>
-          <t>50.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="S18" s="6" t="n">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="T18" s="6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U18" s="6" t="inlineStr">
         <is>
-          <t>0.83%</t>
+          <t>0.00%</t>
         </is>
       </c>
     </row>
@@ -5779,14 +5777,14 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H19" s="6" t="n">
         <v>3</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>186</v>
+        <v>558</v>
       </c>
       <c r="J19" s="6" t="n">
         <v>0</v>
@@ -5797,7 +5795,7 @@
         </is>
       </c>
       <c r="L19" s="6" t="n">
-        <v>1302</v>
+        <v>3906</v>
       </c>
       <c r="M19" s="6" t="n">
         <v>0</v>
@@ -5813,7 +5811,7 @@
         </is>
       </c>
       <c r="P19" s="6" t="n">
-        <v>372</v>
+        <v>1116</v>
       </c>
       <c r="Q19" s="6" t="n">
         <v>0</v>
@@ -5824,7 +5822,7 @@
         </is>
       </c>
       <c r="S19" s="6" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="T19" s="6" t="n">
         <v>0</v>
@@ -5862,14 +5860,14 @@
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H20" s="6" t="n">
         <v>7</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>434</v>
+        <v>1302</v>
       </c>
       <c r="J20" s="6" t="n">
         <v>0</v>
@@ -5880,7 +5878,7 @@
         </is>
       </c>
       <c r="L20" s="6" t="n">
-        <v>3038</v>
+        <v>9114</v>
       </c>
       <c r="M20" s="6" t="n">
         <v>0</v>
@@ -5896,7 +5894,7 @@
         </is>
       </c>
       <c r="P20" s="6" t="n">
-        <v>868</v>
+        <v>2604</v>
       </c>
       <c r="Q20" s="6" t="n">
         <v>0</v>
@@ -5907,7 +5905,7 @@
         </is>
       </c>
       <c r="S20" s="6" t="n">
-        <v>42</v>
+        <v>126</v>
       </c>
       <c r="T20" s="6" t="n">
         <v>0</v>
@@ -5945,14 +5943,14 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H21" s="6" t="n">
         <v>9</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>558</v>
+        <v>1674</v>
       </c>
       <c r="J21" s="6" t="n">
         <v>0</v>
@@ -5963,7 +5961,7 @@
         </is>
       </c>
       <c r="L21" s="6" t="n">
-        <v>3906</v>
+        <v>11718</v>
       </c>
       <c r="M21" s="6" t="n">
         <v>0</v>
@@ -5979,7 +5977,7 @@
         </is>
       </c>
       <c r="P21" s="6" t="n">
-        <v>1116</v>
+        <v>3348</v>
       </c>
       <c r="Q21" s="6" t="n">
         <v>0</v>
@@ -5990,7 +5988,7 @@
         </is>
       </c>
       <c r="S21" s="6" t="n">
-        <v>54</v>
+        <v>162</v>
       </c>
       <c r="T21" s="6" t="n">
         <v>0</v>
@@ -6028,14 +6026,14 @@
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H22" s="6" t="n">
         <v>8</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>496</v>
+        <v>1488</v>
       </c>
       <c r="J22" s="6" t="n">
         <v>0</v>
@@ -6046,7 +6044,7 @@
         </is>
       </c>
       <c r="L22" s="6" t="n">
-        <v>3472</v>
+        <v>10416</v>
       </c>
       <c r="M22" s="6" t="n">
         <v>0</v>
@@ -6062,7 +6060,7 @@
         </is>
       </c>
       <c r="P22" s="6" t="n">
-        <v>992</v>
+        <v>2976</v>
       </c>
       <c r="Q22" s="6" t="n">
         <v>0</v>
@@ -6073,7 +6071,7 @@
         </is>
       </c>
       <c r="S22" s="6" t="n">
-        <v>48</v>
+        <v>144</v>
       </c>
       <c r="T22" s="6" t="n">
         <v>0</v>
@@ -6111,14 +6109,14 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H23" s="6" t="n">
         <v>4</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>248</v>
+        <v>744</v>
       </c>
       <c r="J23" s="6" t="n">
         <v>0</v>
@@ -6129,7 +6127,7 @@
         </is>
       </c>
       <c r="L23" s="6" t="n">
-        <v>1736</v>
+        <v>5208</v>
       </c>
       <c r="M23" s="6" t="n">
         <v>0</v>
@@ -6145,7 +6143,7 @@
         </is>
       </c>
       <c r="P23" s="6" t="n">
-        <v>496</v>
+        <v>1488</v>
       </c>
       <c r="Q23" s="6" t="n">
         <v>0</v>
@@ -6156,7 +6154,7 @@
         </is>
       </c>
       <c r="S23" s="6" t="n">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="T23" s="6" t="n">
         <v>0</v>
@@ -6194,14 +6192,14 @@
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H24" s="6" t="n">
         <v>3</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>186</v>
+        <v>558</v>
       </c>
       <c r="J24" s="6" t="n">
         <v>0</v>
@@ -6212,7 +6210,7 @@
         </is>
       </c>
       <c r="L24" s="6" t="n">
-        <v>1302</v>
+        <v>3906</v>
       </c>
       <c r="M24" s="6" t="n">
         <v>0</v>
@@ -6228,7 +6226,7 @@
         </is>
       </c>
       <c r="P24" s="6" t="n">
-        <v>372</v>
+        <v>1116</v>
       </c>
       <c r="Q24" s="6" t="n">
         <v>0</v>
@@ -6239,7 +6237,7 @@
         </is>
       </c>
       <c r="S24" s="6" t="n">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="T24" s="6" t="n">
         <v>0</v>
@@ -6277,14 +6275,14 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H25" s="6" t="n">
         <v>11</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>682</v>
+        <v>2046</v>
       </c>
       <c r="J25" s="6" t="n">
         <v>0</v>
@@ -6295,7 +6293,7 @@
         </is>
       </c>
       <c r="L25" s="6" t="n">
-        <v>4774</v>
+        <v>14322</v>
       </c>
       <c r="M25" s="6" t="n">
         <v>0</v>
@@ -6311,7 +6309,7 @@
         </is>
       </c>
       <c r="P25" s="6" t="n">
-        <v>1364</v>
+        <v>4092</v>
       </c>
       <c r="Q25" s="6" t="n">
         <v>0</v>
@@ -6322,7 +6320,7 @@
         </is>
       </c>
       <c r="S25" s="6" t="n">
-        <v>66</v>
+        <v>198</v>
       </c>
       <c r="T25" s="6" t="n">
         <v>0</v>
@@ -6360,14 +6358,14 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H26" s="6" t="n">
         <v>15</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>930</v>
+        <v>2790</v>
       </c>
       <c r="J26" s="6" t="n">
         <v>0</v>
@@ -6378,7 +6376,7 @@
         </is>
       </c>
       <c r="L26" s="6" t="n">
-        <v>6510</v>
+        <v>19530</v>
       </c>
       <c r="M26" s="6" t="n">
         <v>0</v>
@@ -6394,7 +6392,7 @@
         </is>
       </c>
       <c r="P26" s="6" t="n">
-        <v>1860</v>
+        <v>5580</v>
       </c>
       <c r="Q26" s="6" t="n">
         <v>0</v>
@@ -6405,7 +6403,7 @@
         </is>
       </c>
       <c r="S26" s="6" t="n">
-        <v>90</v>
+        <v>270</v>
       </c>
       <c r="T26" s="6" t="n">
         <v>0</v>
@@ -6443,14 +6441,14 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H27" s="6" t="n">
         <v>4</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>248</v>
+        <v>744</v>
       </c>
       <c r="J27" s="6" t="n">
         <v>0</v>
@@ -6461,7 +6459,7 @@
         </is>
       </c>
       <c r="L27" s="6" t="n">
-        <v>1736</v>
+        <v>5208</v>
       </c>
       <c r="M27" s="6" t="n">
         <v>0</v>
@@ -6477,7 +6475,7 @@
         </is>
       </c>
       <c r="P27" s="6" t="n">
-        <v>496</v>
+        <v>1488</v>
       </c>
       <c r="Q27" s="6" t="n">
         <v>0</v>
@@ -6488,7 +6486,7 @@
         </is>
       </c>
       <c r="S27" s="6" t="n">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="T27" s="6" t="n">
         <v>0</v>
@@ -6526,14 +6524,14 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H28" s="6" t="n">
         <v>5</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>310</v>
+        <v>930</v>
       </c>
       <c r="J28" s="6" t="n">
         <v>0</v>
@@ -6544,7 +6542,7 @@
         </is>
       </c>
       <c r="L28" s="6" t="n">
-        <v>2170</v>
+        <v>6510</v>
       </c>
       <c r="M28" s="6" t="n">
         <v>0</v>
@@ -6560,7 +6558,7 @@
         </is>
       </c>
       <c r="P28" s="6" t="n">
-        <v>620</v>
+        <v>1860</v>
       </c>
       <c r="Q28" s="6" t="n">
         <v>0</v>
@@ -6571,7 +6569,7 @@
         </is>
       </c>
       <c r="S28" s="6" t="n">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="T28" s="6" t="n">
         <v>0</v>
@@ -6609,14 +6607,14 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H29" s="6" t="n">
         <v>12</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>744</v>
+        <v>2232</v>
       </c>
       <c r="J29" s="6" t="n">
         <v>0</v>
@@ -6627,7 +6625,7 @@
         </is>
       </c>
       <c r="L29" s="6" t="n">
-        <v>5208</v>
+        <v>15624</v>
       </c>
       <c r="M29" s="6" t="n">
         <v>0</v>
@@ -6643,7 +6641,7 @@
         </is>
       </c>
       <c r="P29" s="6" t="n">
-        <v>1488</v>
+        <v>4464</v>
       </c>
       <c r="Q29" s="6" t="n">
         <v>0</v>
@@ -6654,7 +6652,7 @@
         </is>
       </c>
       <c r="S29" s="6" t="n">
-        <v>72</v>
+        <v>216</v>
       </c>
       <c r="T29" s="6" t="n">
         <v>0</v>
@@ -6692,14 +6690,14 @@
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H30" s="6" t="n">
         <v>8</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>496</v>
+        <v>1488</v>
       </c>
       <c r="J30" s="6" t="n">
         <v>0</v>
@@ -6710,7 +6708,7 @@
         </is>
       </c>
       <c r="L30" s="6" t="n">
-        <v>3472</v>
+        <v>10416</v>
       </c>
       <c r="M30" s="6" t="n">
         <v>0</v>
@@ -6726,7 +6724,7 @@
         </is>
       </c>
       <c r="P30" s="6" t="n">
-        <v>992</v>
+        <v>2976</v>
       </c>
       <c r="Q30" s="6" t="n">
         <v>0</v>
@@ -6737,7 +6735,7 @@
         </is>
       </c>
       <c r="S30" s="6" t="n">
-        <v>48</v>
+        <v>144</v>
       </c>
       <c r="T30" s="6" t="n">
         <v>0</v>
@@ -6775,14 +6773,14 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H31" s="6" t="n">
         <v>4</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>248</v>
+        <v>744</v>
       </c>
       <c r="J31" s="6" t="n">
         <v>0</v>
@@ -6793,7 +6791,7 @@
         </is>
       </c>
       <c r="L31" s="6" t="n">
-        <v>1736</v>
+        <v>5208</v>
       </c>
       <c r="M31" s="6" t="n">
         <v>0</v>
@@ -6809,7 +6807,7 @@
         </is>
       </c>
       <c r="P31" s="6" t="n">
-        <v>496</v>
+        <v>1488</v>
       </c>
       <c r="Q31" s="6" t="n">
         <v>0</v>
@@ -6820,7 +6818,7 @@
         </is>
       </c>
       <c r="S31" s="6" t="n">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="T31" s="6" t="n">
         <v>0</v>
@@ -6858,14 +6856,14 @@
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H32" s="6" t="n">
         <v>14</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>868</v>
+        <v>2604</v>
       </c>
       <c r="J32" s="6" t="n">
         <v>0</v>
@@ -6876,7 +6874,7 @@
         </is>
       </c>
       <c r="L32" s="6" t="n">
-        <v>6076</v>
+        <v>18228</v>
       </c>
       <c r="M32" s="6" t="n">
         <v>0</v>
@@ -6892,7 +6890,7 @@
         </is>
       </c>
       <c r="P32" s="6" t="n">
-        <v>1736</v>
+        <v>5208</v>
       </c>
       <c r="Q32" s="6" t="n">
         <v>0</v>
@@ -6903,7 +6901,7 @@
         </is>
       </c>
       <c r="S32" s="6" t="n">
-        <v>84</v>
+        <v>252</v>
       </c>
       <c r="T32" s="6" t="n">
         <v>0</v>
@@ -6941,14 +6939,14 @@
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H33" s="6" t="n">
         <v>4</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>248</v>
+        <v>744</v>
       </c>
       <c r="J33" s="6" t="n">
         <v>0</v>
@@ -6959,7 +6957,7 @@
         </is>
       </c>
       <c r="L33" s="6" t="n">
-        <v>1736</v>
+        <v>5208</v>
       </c>
       <c r="M33" s="6" t="n">
         <v>0</v>
@@ -6975,7 +6973,7 @@
         </is>
       </c>
       <c r="P33" s="6" t="n">
-        <v>496</v>
+        <v>1488</v>
       </c>
       <c r="Q33" s="6" t="n">
         <v>0</v>
@@ -6986,7 +6984,7 @@
         </is>
       </c>
       <c r="S33" s="6" t="n">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="T33" s="6" t="n">
         <v>0</v>
@@ -7024,14 +7022,14 @@
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H34" s="6" t="n">
         <v>2</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>124</v>
+        <v>372</v>
       </c>
       <c r="J34" s="6" t="n">
         <v>0</v>
@@ -7042,7 +7040,7 @@
         </is>
       </c>
       <c r="L34" s="6" t="n">
-        <v>868</v>
+        <v>2604</v>
       </c>
       <c r="M34" s="6" t="n">
         <v>0</v>
@@ -7058,7 +7056,7 @@
         </is>
       </c>
       <c r="P34" s="6" t="n">
-        <v>248</v>
+        <v>744</v>
       </c>
       <c r="Q34" s="6" t="n">
         <v>0</v>
@@ -7069,7 +7067,7 @@
         </is>
       </c>
       <c r="S34" s="6" t="n">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="T34" s="6" t="n">
         <v>0</v>
@@ -7107,14 +7105,14 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>0 از 2</t>
+          <t>0 از 6</t>
         </is>
       </c>
       <c r="H35" s="6" t="n">
         <v>4</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>248</v>
+        <v>744</v>
       </c>
       <c r="J35" s="6" t="n">
         <v>0</v>
@@ -7125,7 +7123,7 @@
         </is>
       </c>
       <c r="L35" s="6" t="n">
-        <v>1736</v>
+        <v>5208</v>
       </c>
       <c r="M35" s="6" t="n">
         <v>0</v>
@@ -7141,7 +7139,7 @@
         </is>
       </c>
       <c r="P35" s="6" t="n">
-        <v>496</v>
+        <v>1488</v>
       </c>
       <c r="Q35" s="6" t="n">
         <v>0</v>
@@ -7152,7 +7150,7 @@
         </is>
       </c>
       <c r="S35" s="6" t="n">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="T35" s="6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Fix multi-folder evaluation and district detection for Golpayegan reports
- Re-architect calculate_period_scores.py with modular, robust architecture
- Implement universal Excel workbook loader supporting .xlsx, .xlsm, binary .xls (via xlrd), and HTML tables
- Add deep Unicode normalization (handling Arabic/Persian kaf/yeh, zero-width chars, tatweel, and Windows LTR/RTL marks)
- Make path and folder discovery foolproof across script_dir and cwd
- Refine attendance column identification to avoid misidentifying audience type headers
- Add Sheet 3 (Audit Trail) to نمرات_نهایی_نواحی.xlsx for complete file processing transparency
- Update packages (scores_package.zip and nasra_full_package.zip) and documentation

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/نمرات_نهایی_نواحی.xlsx
+++ b/نمرات_نهایی_نواحی.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="فقط نام و نمره (ساده)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="مقایسه دو مقیاس" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="پایش فایل‌های ورودی" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +31,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -48,7 +49,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001E3A8A"/>
-      <sz val="15"/>
+      <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -62,7 +63,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -93,6 +94,18 @@
         <bgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00374151"/>
+        <bgColor rgb="00374151"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -120,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -151,6 +164,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -783,7 +802,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>12.9</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27">
@@ -1803,10 +1822,10 @@
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>12.9</v>
+        <v>43</v>
       </c>
       <c r="D28" s="8" t="n">
-        <v>73.90000000000001</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
@@ -1818,7 +1837,7 @@
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>12.9%</t>
+          <t>43.0%</t>
         </is>
       </c>
       <c r="H28" s="10" t="inlineStr">
@@ -2085,4 +2104,248 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>گزارش وضعیت شناسایی، استخراج و پردازش تک‌تک فایل‌های اکسل در سیستم</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>ردیف</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>نام فایل</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>پوشه / برچسب</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>ماه منتسب</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>ناحیه شناسایی‌شده</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>روش شناسایی</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>حضوری</t>
+        </is>
+      </c>
+      <c r="H3" s="11" t="inlineStr">
+        <is>
+          <t>مجازی</t>
+        </is>
+      </c>
+      <c r="I3" s="11" t="inlineStr">
+        <is>
+          <t>خلاقانه</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>تولیدات</t>
+        </is>
+      </c>
+      <c r="K3" s="11" t="inlineStr">
+        <is>
+          <t>وضعیت</t>
+        </is>
+      </c>
+      <c r="L3" s="11" t="inlineStr">
+        <is>
+          <t>پیام خطا / توضیحات</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>گلپایگان.xlsx</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>تیر</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>تیر</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>گلپایگان</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>نام فایل</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>500</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>موفق</t>
+        </is>
+      </c>
+      <c r="L4" s="10" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>گلپایگان.xlsx</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>مرداد</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>مرداد</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>گلپایگان</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>نام فایل</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>500</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>موفق</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>گلپایگان.xlsx</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>شهریور</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>شهریور</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>گلپایگان</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>نام فایل</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>500</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>موفق</t>
+        </is>
+      </c>
+      <c r="L6" s="10" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add threaded 10s per-file timeout, QuickEdit protection, auto-startfile and enhanced bat runners
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/نمرات_نهایی_نواحی.xlsx
+++ b/نمرات_نهایی_نواحی.xlsx
@@ -133,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -169,6 +169,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2112,7 +2115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2257,12 +2260,12 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>مرداد</t>
+          <t>شهریور</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>مرداد</t>
+          <t>شهریور</t>
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -2305,12 +2308,12 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>شهریور</t>
+          <t>مرداد</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>شهریور</t>
+          <t>مرداد</t>
         </is>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -2341,6 +2344,58 @@
         </is>
       </c>
       <c r="L6" s="10" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>test.xls</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>پوشه اصلی برنامه</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>خطا</t>
+        </is>
+      </c>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>جهت پردازش فایل باینری قدیمی .xls نصب پکیج xlrd الزامی است.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Switch to ultra-fast in-memory streaming read_only mode, remove thread pool bottlenecks, and silence openpyxl warnings
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/نمرات_نهایی_نواحی.xlsx
+++ b/نمرات_نهایی_نواحی.xlsx
@@ -133,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -169,9 +169,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2115,7 +2112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2345,58 +2342,6 @@
       </c>
       <c r="L6" s="10" t="inlineStr"/>
     </row>
-    <row r="7">
-      <c r="A7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>test.xls</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>پوشه اصلی برنامه</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E7" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="13" t="inlineStr">
-        <is>
-          <t>خطا</t>
-        </is>
-      </c>
-      <c r="L7" s="10" t="inlineStr">
-        <is>
-          <t>جهت پردازش فایل باینری قدیمی .xls نصب پکیج xlrd الزامی است.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>

</xml_diff>